<commit_message>
The commit-count check was self-defeating, and a second stale count
check_consistency.py compared the methods form's commit count against HEAD
exactly, which can never hold: committing the fix increments the number it
just fixed. A file recording the repository's own commit count is correct only
up to the commit that writes it, so the check now allows a lag of exactly one
and no more.

Widening the match from the first occurrence to all of them found a second
stale figure: the Track 1 effort answer also said 32 commits. Both now read 40.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/submissions/methods_description_gummietech.xlsx
+++ b/submissions/methods_description_gummietech.xlsx
@@ -682,7 +682,7 @@
 The full pipeline runs in **under 10 minutes end to end** on a 2019-class laptop (8 GB RAM,
 8 cores), dominated by Ensembl VEP REST latency, not compute. Standard library Python only,
 no cluster, no paid compute. **The analysis time is the cost**: the work spans 2026-08-31
-to 2026-09-04 across 32 commits, the large majority of it verification and audit rather
+to 2026-09-04 across 40 commits, the large majority of it verification and audit rather
 than the initial pipeline, which was the smaller part of the effort.
 ### Method abstract (≤500 words)
 We recover a compound-heterozygous BUB1B candidate — `p.Leu737Ter` (ClinVar
@@ -831,7 +831,7 @@
       </c>
       <c r="B18" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">The full pipeline runs in under 10 minutes end to end on a 2019-class laptop (8 GB RAM, 8 cores), dominated by Ensembl VEP REST latency, not compute. Standard library Python only, no cluster, no paid compute. The analysis time is the cost: the work spans 2026-08-31 to 2026-09-04 across 32 commits, the large majority of it verification and audit rather than the initial pipeline, which was the smaller part of the effort.</t>
+          <t xml:space="preserve">The full pipeline runs in under 10 minutes end to end on a 2019-class laptop (8 GB RAM, 8 cores), dominated by Ensembl VEP REST latency, not compute. Standard library Python only, no cluster, no paid compute. The analysis time is the cost: the work spans 2026-08-31 to 2026-09-04 across 40 commits, the large majority of it verification and audit rather than the initial pipeline, which was the smaller part of the effort.</t>
         </is>
       </c>
     </row>
@@ -984,7 +984,7 @@
   buried than Asn1002. That is reported as the result it is, and the report's Limitation 1
   is tightened rather than relaxed.
 ### Time or effort
-2026-08-31 to 2026-09-04, 39 commits. The mechanism characterisation and the verification
+2026-08-31 to 2026-09-04, 40 commits. The mechanism characterisation and the verification
 passes consumed substantially more effort than the drug search itself, which is the correct
 ratio for this problem: the search is cheap and the reframing is what makes it point
 anywhere useful.
@@ -1129,7 +1129,7 @@
       </c>
       <c r="B16" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-08-31 to 2026-09-04, 39 commits. The mechanism characterisation and the verification passes consumed substantially more effort than the drug search itself, which is the correct ratio for this problem: the search is cheap and the reframing is what makes it point anywhere useful.</t>
+          <t xml:space="preserve">2026-08-31 to 2026-09-04, 40 commits. The mechanism characterisation and the verification passes consumed substantially more effort than the drug search itself, which is the correct ratio for this problem: the search is cheap and the reframing is what makes it point anywhere useful.</t>
         </is>
       </c>
     </row>

</xml_diff>